<commit_message>
blank_rows test had requested missing channel
the summarise biotek data doesn't have all of the channels that are in the normal biotek data file
</commit_message>
<xml_diff>
--- a/test/inputs/blank_rows.xlsx
+++ b/test/inputs/blank_rows.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0C2FC0-FCCA-084A-B6FC-FB358B7C9888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0628626A-A127-B64E-B092-09BA77A93EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30240" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="-30240" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
   <si>
     <t>Plate</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>OD_600</t>
+  </si>
+  <si>
+    <t>OD_600, OD_700, GFP_485_530</t>
   </si>
 </sst>
 </file>
@@ -563,7 +566,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>

</xml_diff>